<commit_message>
Update lead-sample.xlsx and add temporary file for tracking changes
</commit_message>
<xml_diff>
--- a/public/lead-sample.xlsx
+++ b/public/lead-sample.xlsx
@@ -8,20 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\AWX Platform\autoworx-platform\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{000B4A1A-920A-4950-988B-1A5D9C44B206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3535FFB0-E027-4DDC-BE89-1C0809935F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
-    </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
@@ -36,7 +33,7 @@
     <t>email</t>
   </si>
   <si>
-    <t>contactNumber</t>
+    <t>contact</t>
   </si>
   <si>
     <t>vehicle(year-make-model)</t>
@@ -55,38 +52,29 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <charset val="1"/>
     </font>
     <font>
       <u/>
       <sz val="10"/>
-      <color theme="10"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -121,92 +109,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF9A9A9A"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -271,45 +188,49 @@
         <a:cs typeface="Arial"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme>
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
                 <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
                 <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
                 <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
         </a:gradFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
                 <a:lumMod val="102000"/>
                 <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
                 <a:lumMod val="100000"/>
                 <a:shade val="100000"/>
               </a:schemeClr>
@@ -317,24 +238,33 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
                 <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
@@ -347,7 +277,13 @@
           <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -357,13 +293,15 @@
         <a:solidFill>
           <a:schemeClr val="phClr">
             <a:tint val="95000"/>
+            <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
+                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
               </a:schemeClr>
@@ -371,6 +309,7 @@
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
+                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
               </a:schemeClr>
@@ -378,11 +317,11 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -395,12 +334,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
-    <outlinePr summaryBelow="0"/>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="2" max="2" width="29" customWidth="1"/>
     <col min="4" max="4" width="27.5703125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -426,7 +365,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
-      <c r="B2" s="5"/>
+      <c r="B2" s="3"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
@@ -489,7 +428,6 @@
       <c r="F9" s="4"/>
     </row>
   </sheetData>
-  <pageMargins left="0.74791666666666701" right="0.74791666666666701" top="0.98402777777777795" bottom="0.98402777777777795" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: update lead-sample.xlsx with new data
</commit_message>
<xml_diff>
--- a/public/lead-sample.xlsx
+++ b/public/lead-sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\AWX Platform\autoworx-platform\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3535FFB0-E027-4DDC-BE89-1C0809935F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D04DB9BE-08D7-4542-9DF8-1B4233F8BEB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
     <t>source</t>
   </si>
   <si>
-    <t>created_at</t>
+    <t>created_at(mm/dd/yyyy hr:min:sec)</t>
   </si>
 </sst>
 </file>
@@ -341,6 +341,7 @@
   <cols>
     <col min="2" max="2" width="29" customWidth="1"/>
     <col min="4" max="4" width="27.5703125" customWidth="1"/>
+    <col min="6" max="6" width="30.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>